<commit_message>
Commit 4: updated the schematic
Added crystal load capacitors, test points, SWO for debugging, PB8 as boot/CAN_RX, Pi filter on VDDA, and noted peripherals.
</commit_message>
<xml_diff>
--- a/ThreeShuntFocBoard/STM32G431C6_PIN_Selection_details.xlsx
+++ b/ThreeShuntFocBoard/STM32G431C6_PIN_Selection_details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BLDC\Git\Implementations\TransistorDrivenInverter\ThreeShuntFocBoard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C462D0C2-4ACF-4A0B-BDEA-A44BCE2EE8D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF853CF1-0B5C-4269-A2FE-7E69705BE33C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{790DF44D-2C80-4A51-A3F0-1B22F97E8EFE}"/>
   </bookViews>
@@ -1182,7 +1182,7 @@
     <col min="2" max="2" width="70.33203125" style="4" customWidth="1"/>
     <col min="3" max="3" width="51.77734375" style="31" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.33203125" style="51" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="84.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1202,7 +1202,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A2" s="33">
         <v>1</v>
       </c>
@@ -1217,7 +1217,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" s="34">
         <v>2</v>
       </c>
@@ -1228,7 +1228,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="50"/>
-      <c r="F3" t="s">
+      <c r="F3" s="14" t="s">
         <v>104</v>
       </c>
     </row>

</xml_diff>